<commit_message>
feat: release da versão definitiva do Extrator de Diárias V2
Central Analítica (Sprints 17-19) homologada definitivamente em
2026-08-04: pesquisa/filtros sobre a Base Local SQLite, Dashboard,
Relatórios exportáveis (PDF/Excel/CSV) e Diagnóstico automático do
recorte filtrado. Documentação, screenshots e GIF de demonstração
atualizados para refletir exclusivamente a versão definitiva.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/demo/planilha_demo.xlsx
+++ b/scripts/demo/planilha_demo.xlsx
@@ -502,6 +502,31 @@
           <t>MOTIVO</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>VALOR DA PASSAGEM</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>QUANT. DIÁRIA INTEGRAL</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>QUANT. DIÁRIA PARCIAL</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>VALOR TOTAL DAS DIÁRIAS</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>LOCAL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">

</xml_diff>